<commit_message>
added google maps link to plot and changed format slightly
</commit_message>
<xml_diff>
--- a/results/tgt_2026_segment_analysis.xlsx
+++ b/results/tgt_2026_segment_analysis.xlsx
@@ -483,7 +483,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>START</t>
+          <t>START (奥多摩運動公園)</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -819,7 +819,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>FINISH</t>
+          <t>FINISH (奥多摩運動公園)</t>
         </is>
       </c>
       <c r="B14" t="n">

</xml_diff>

<commit_message>
add different ways of calculating time
</commit_message>
<xml_diff>
--- a/results/tgt_2026_segment_analysis.xlsx
+++ b/results/tgt_2026_segment_analysis.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segment Statistics" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Race Plan (target_time)" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -518,22 +519,22 @@
         <v>7.5</v>
       </c>
       <c r="C3" t="n">
-        <v>667.0162543172806</v>
+        <v>661.8797463188054</v>
       </c>
       <c r="D3" t="n">
-        <v>947.1397806680607</v>
+        <v>942.8824897693294</v>
       </c>
       <c r="E3" t="n">
         <v>7.5</v>
       </c>
       <c r="F3" t="n">
-        <v>945.4603658489441</v>
+        <v>942.8824897693294</v>
       </c>
       <c r="G3" t="n">
-        <v>665.0635263507801</v>
+        <v>665.9427434505239</v>
       </c>
       <c r="H3" t="n">
-        <v>12.60613821131925</v>
+        <v>12.57176653025772</v>
       </c>
     </row>
     <row r="4">
@@ -546,22 +547,22 @@
         <v>19.3</v>
       </c>
       <c r="C4" t="n">
-        <v>286.0992944929012</v>
+        <v>285.4917155135353</v>
       </c>
       <c r="D4" t="n">
-        <v>1682.260133310758</v>
+        <v>1683.866521793493</v>
       </c>
       <c r="E4" t="n">
         <v>11.8</v>
       </c>
       <c r="F4" t="n">
-        <v>736.7997674618164</v>
+        <v>740.8559307881177</v>
       </c>
       <c r="G4" t="n">
-        <v>1116.037312467079</v>
+        <v>1117.372062829435</v>
       </c>
       <c r="H4" t="n">
-        <v>6.244065825947597</v>
+        <v>6.278440091424726</v>
       </c>
     </row>
     <row r="5">
@@ -574,22 +575,22 @@
         <v>28</v>
       </c>
       <c r="C5" t="n">
-        <v>244.1405543582715</v>
+        <v>270.2025177162001</v>
       </c>
       <c r="D5" t="n">
-        <v>2316.037458238309</v>
+        <v>2325.029709396688</v>
       </c>
       <c r="E5" t="n">
         <v>8.699999999999999</v>
       </c>
       <c r="F5" t="n">
-        <v>633.7773249275515</v>
+        <v>641.2912888392384</v>
       </c>
       <c r="G5" t="n">
-        <v>674.6593652559289</v>
+        <v>656.4523854005267</v>
       </c>
       <c r="H5" t="n">
-        <v>7.284796838247718</v>
+        <v>7.371164239531476</v>
       </c>
     </row>
     <row r="6">
@@ -602,22 +603,22 @@
         <v>45</v>
       </c>
       <c r="C6" t="n">
-        <v>226.9307344330622</v>
+        <v>228.2608106972169</v>
       </c>
       <c r="D6" t="n">
-        <v>3357.56816580374</v>
+        <v>3373.182701102885</v>
       </c>
       <c r="E6" t="n">
         <v>17</v>
       </c>
       <c r="F6" t="n">
-        <v>1041.530707565443</v>
+        <v>1048.152991706207</v>
       </c>
       <c r="G6" t="n">
-        <v>1059.713908379867</v>
+        <v>1090.09469872519</v>
       </c>
       <c r="H6" t="n">
-        <v>6.126651220973196</v>
+        <v>6.165605833565923</v>
       </c>
     </row>
     <row r="7">
@@ -630,22 +631,22 @@
         <v>59</v>
       </c>
       <c r="C7" t="n">
-        <v>198.2795229117985</v>
+        <v>195.8715224255816</v>
       </c>
       <c r="D7" t="n">
-        <v>4057.511553711809</v>
+        <v>4074.790603809976</v>
       </c>
       <c r="E7" t="n">
         <v>14</v>
       </c>
       <c r="F7" t="n">
-        <v>699.7515192389917</v>
+        <v>701.607902707103</v>
       </c>
       <c r="G7" t="n">
-        <v>728.6979183463775</v>
+        <v>733.9971909787382</v>
       </c>
       <c r="H7" t="n">
-        <v>4.998225137421369</v>
+        <v>5.01148501933645</v>
       </c>
     </row>
     <row r="8">
@@ -658,22 +659,22 @@
         <v>71</v>
       </c>
       <c r="C8" t="n">
-        <v>216.2894414977829</v>
+        <v>211.8587872207498</v>
       </c>
       <c r="D8" t="n">
-        <v>4823.729233080529</v>
+        <v>4840.964655488125</v>
       </c>
       <c r="E8" t="n">
         <v>12</v>
       </c>
       <c r="F8" t="n">
-        <v>766.4095480378079</v>
+        <v>766.1740516781615</v>
       </c>
       <c r="G8" t="n">
-        <v>748.2077607827393</v>
+        <v>750.1867868829933</v>
       </c>
       <c r="H8" t="n">
-        <v>6.386746233648399</v>
+        <v>6.384783763984679</v>
       </c>
     </row>
     <row r="9">
@@ -686,22 +687,22 @@
         <v>88.5</v>
       </c>
       <c r="C9" t="n">
-        <v>305.270352391576</v>
+        <v>315.0548541845947</v>
       </c>
       <c r="D9" t="n">
-        <v>6289.040751615353</v>
+        <v>6314.372494909166</v>
       </c>
       <c r="E9" t="n">
         <v>17.5</v>
       </c>
       <c r="F9" t="n">
-        <v>1465.311518534781</v>
+        <v>1473.407839421042</v>
       </c>
       <c r="G9" t="n">
-        <v>1376.330607640988</v>
+        <v>1370.211772457197</v>
       </c>
       <c r="H9" t="n">
-        <v>8.373208677341603</v>
+        <v>8.419473368120238</v>
       </c>
     </row>
     <row r="10">
@@ -714,22 +715,22 @@
         <v>100.8</v>
       </c>
       <c r="C10" t="n">
-        <v>204.7677653851742</v>
+        <v>201.35</v>
       </c>
       <c r="D10" t="n">
-        <v>7062.297042031661</v>
+        <v>7087.718351684849</v>
       </c>
       <c r="E10" t="n">
         <v>12.3</v>
       </c>
       <c r="F10" t="n">
-        <v>773.2562904163076</v>
+        <v>773.345856775705</v>
       </c>
       <c r="G10" t="n">
-        <v>873.7588774227092</v>
+        <v>887.0507109602997</v>
       </c>
       <c r="H10" t="n">
-        <v>6.286636507449657</v>
+        <v>6.287364689233375</v>
       </c>
     </row>
     <row r="11">
@@ -742,22 +743,22 @@
         <v>117.9</v>
       </c>
       <c r="C11" t="n">
-        <v>699.8042343269917</v>
+        <v>718.4395719536392</v>
       </c>
       <c r="D11" t="n">
-        <v>8188.674301135295</v>
+        <v>8209.14465729939</v>
       </c>
       <c r="E11" t="n">
         <v>17.10000000000001</v>
       </c>
       <c r="F11" t="n">
-        <v>1125.660036455141</v>
+        <v>1121.426305614531</v>
       </c>
       <c r="G11" t="n">
-        <v>631.3407901618173</v>
+        <v>603.3959060859178</v>
       </c>
       <c r="H11" t="n">
-        <v>6.582807230731818</v>
+        <v>6.558048570845208</v>
       </c>
     </row>
     <row r="12">
@@ -770,22 +771,22 @@
         <v>134.8</v>
       </c>
       <c r="C12" t="n">
-        <v>220.375586408151</v>
+        <v>228.6285740986007</v>
       </c>
       <c r="D12" t="n">
-        <v>9005.747932390315</v>
+        <v>9037.894441375362</v>
       </c>
       <c r="E12" t="n">
         <v>16.90000000000001</v>
       </c>
       <c r="F12" t="n">
-        <v>816.8299327447622</v>
+        <v>828.7497840759515</v>
       </c>
       <c r="G12" t="n">
-        <v>1296.502279173818</v>
+        <v>1319.501609505964</v>
       </c>
       <c r="H12" t="n">
-        <v>4.833313211507466</v>
+        <v>4.90384487618906</v>
       </c>
     </row>
     <row r="13">
@@ -798,22 +799,22 @@
         <v>152.9</v>
       </c>
       <c r="C13" t="n">
-        <v>625.8594161020432</v>
+        <v>679.1060519944383</v>
       </c>
       <c r="D13" t="n">
-        <v>10731.33941252795</v>
+        <v>10782.04113579533</v>
       </c>
       <c r="E13" t="n">
         <v>18.09999999999999</v>
       </c>
       <c r="F13" t="n">
-        <v>1726.552401296333</v>
+        <v>1744.14669441999</v>
       </c>
       <c r="G13" t="n">
-        <v>1320.107650443733</v>
+        <v>1293.162599472007</v>
       </c>
       <c r="H13" t="n">
-        <v>9.538963543073669</v>
+        <v>9.636169582430885</v>
       </c>
     </row>
     <row r="14">
@@ -826,22 +827,690 @@
         <v>158.8</v>
       </c>
       <c r="C14" t="n">
-        <v>384.02</v>
+        <v>345.4817763220301</v>
       </c>
       <c r="D14" t="n">
-        <v>10831.97666992459</v>
+        <v>10841.43545225183</v>
       </c>
       <c r="E14" t="n">
         <v>5.900000000000006</v>
       </c>
       <c r="F14" t="n">
-        <v>100.6372573966486</v>
+        <v>59.39431645649455</v>
       </c>
       <c r="G14" t="n">
-        <v>342.4766734986917</v>
+        <v>393.4891958525554</v>
       </c>
       <c r="H14" t="n">
-        <v>1.705716227061839</v>
+        <v>1.006683329771093</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Point Name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Total Distance (km)</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Elevation (m)</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Accum. Elevation Gain (m)</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Segment Distance (km)</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Segment Elevation Gain (m)</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Segment Elevation Loss (m)</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Segment Running Time</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Stop Time</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Elapsed Time</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>START (奥多摩運動公園)</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" t="n">
+        <v>384.9</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>0:00:00</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>0:00:00</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>0:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>CP1 Daikon-yama no Kami (大根山の神)</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="C3" t="n">
+        <v>661.9</v>
+      </c>
+      <c r="D3" t="n">
+        <v>943</v>
+      </c>
+      <c r="E3" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="F3" t="n">
+        <v>943</v>
+      </c>
+      <c r="G3" t="n">
+        <v>666</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>1:50:08</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>0:01:00</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>1:51:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Kawai (川井)</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>19.3</v>
+      </c>
+      <c r="C4" t="n">
+        <v>285.5</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1684</v>
+      </c>
+      <c r="E4" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="F4" t="n">
+        <v>741</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1117</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2:15:46</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>0:02:00</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>4:08:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>A1 Mitake Aid (御岳エイド)</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>28</v>
+      </c>
+      <c r="C5" t="n">
+        <v>270.2</v>
+      </c>
+      <c r="D5" t="n">
+        <v>2325</v>
+      </c>
+      <c r="E5" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="F5" t="n">
+        <v>641</v>
+      </c>
+      <c r="G5" t="n">
+        <v>656</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>1:41:25</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>0:03:00</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>5:53:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>CP2 Umegou (梅郷地区)</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>45</v>
+      </c>
+      <c r="C6" t="n">
+        <v>228.3</v>
+      </c>
+      <c r="D6" t="n">
+        <v>3373</v>
+      </c>
+      <c r="E6" t="n">
+        <v>17</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1048</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1090</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>3:01:36</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>0:03:00</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>8:57:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Hinode Oguno 7-eleven</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>59</v>
+      </c>
+      <c r="C7" t="n">
+        <v>195.9</v>
+      </c>
+      <c r="D7" t="n">
+        <v>4075</v>
+      </c>
+      <c r="E7" t="n">
+        <v>14</v>
+      </c>
+      <c r="F7" t="n">
+        <v>702</v>
+      </c>
+      <c r="G7" t="n">
+        <v>734</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2:17:39</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>0:02:00</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>11:17:35</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>A2 Jurigi (1) (十里木)</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>71</v>
+      </c>
+      <c r="C8" t="n">
+        <v>211.9</v>
+      </c>
+      <c r="D8" t="n">
+        <v>4841</v>
+      </c>
+      <c r="E8" t="n">
+        <v>12</v>
+      </c>
+      <c r="F8" t="n">
+        <v>766</v>
+      </c>
+      <c r="G8" t="n">
+        <v>750</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2:10:21</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>0:05:00</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>13:32:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>A3 Sanogawa (佐野川)</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>88.5</v>
+      </c>
+      <c r="C9" t="n">
+        <v>315.1</v>
+      </c>
+      <c r="D9" t="n">
+        <v>6314</v>
+      </c>
+      <c r="E9" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1473</v>
+      </c>
+      <c r="G9" t="n">
+        <v>1370</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>3:32:48</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>0:02:00</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>17:07:44</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>A4 Fujimi chaya (富士見茶屋)</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>100.8</v>
+      </c>
+      <c r="C10" t="n">
+        <v>201.4</v>
+      </c>
+      <c r="D10" t="n">
+        <v>7088</v>
+      </c>
+      <c r="E10" t="n">
+        <v>12.3</v>
+      </c>
+      <c r="F10" t="n">
+        <v>773</v>
+      </c>
+      <c r="G10" t="n">
+        <v>887</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>2:16:16</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>0:01:30</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>19:25:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Wada-toge (和田峠)</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>117.9</v>
+      </c>
+      <c r="C11" t="n">
+        <v>718.4</v>
+      </c>
+      <c r="D11" t="n">
+        <v>8209</v>
+      </c>
+      <c r="E11" t="n">
+        <v>17.1</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1121</v>
+      </c>
+      <c r="G11" t="n">
+        <v>603</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2:54:08</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>0:02:00</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>22:21:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>A6 Jurigi (2) (十里木)</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>134.8</v>
+      </c>
+      <c r="C12" t="n">
+        <v>228.6</v>
+      </c>
+      <c r="D12" t="n">
+        <v>9038</v>
+      </c>
+      <c r="E12" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="F12" t="n">
+        <v>829</v>
+      </c>
+      <c r="G12" t="n">
+        <v>1320</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>2:54:51</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>0:01:30</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>25:17:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Tomin no mori (都民の森)</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>152.9</v>
+      </c>
+      <c r="C13" t="n">
+        <v>679.1</v>
+      </c>
+      <c r="D13" t="n">
+        <v>10782</v>
+      </c>
+      <c r="E13" t="n">
+        <v>18.1</v>
+      </c>
+      <c r="F13" t="n">
+        <v>1744</v>
+      </c>
+      <c r="G13" t="n">
+        <v>1293</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>3:49:16</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>0:01:30</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>29:08:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>FINISH (奥多摩運動公園)</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>158.8</v>
+      </c>
+      <c r="C14" t="n">
+        <v>345.5</v>
+      </c>
+      <c r="D14" t="n">
+        <v>10841</v>
+      </c>
+      <c r="E14" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="F14" t="n">
+        <v>59</v>
+      </c>
+      <c r="G14" t="n">
+        <v>393</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>0:44:47</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>0:00:00</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>29:53:32</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Planning mode</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>target_time</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Athlete</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Carlos</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Total running time</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>29:29:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Total stop time</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>0:24:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Total finish time</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>29:53:32</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Predicted ITRA score</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>804</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
small edits to athlete
</commit_message>
<xml_diff>
--- a/results/tgt_2026_segment_analysis.xlsx
+++ b/results/tgt_2026_segment_analysis.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segment Statistics" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Race Plan (target_time)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Race Plan (athlete_pb)" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -989,7 +989,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1:50:08</t>
+          <t>1:29:20</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -999,7 +999,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>1:51:08</t>
+          <t>1:30:20</t>
         </is>
       </c>
     </row>
@@ -1029,7 +1029,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2:15:46</t>
+          <t>1:50:21</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -1039,7 +1039,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>4:08:54</t>
+          <t>3:22:41</t>
         </is>
       </c>
     </row>
@@ -1069,7 +1069,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>1:41:25</t>
+          <t>1:21:58</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -1079,7 +1079,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>5:53:19</t>
+          <t>4:47:39</t>
         </is>
       </c>
     </row>
@@ -1109,7 +1109,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>3:01:36</t>
+          <t>2:25:38</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>8:57:56</t>
+          <t>7:16:17</t>
         </is>
       </c>
     </row>
@@ -1149,7 +1149,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2:17:39</t>
+          <t>1:49:56</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -1159,7 +1159,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>11:17:35</t>
+          <t>9:08:13</t>
         </is>
       </c>
     </row>
@@ -1189,7 +1189,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2:10:21</t>
+          <t>1:44:51</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1199,7 +1199,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>13:32:56</t>
+          <t>10:58:04</t>
         </is>
       </c>
     </row>
@@ -1229,7 +1229,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>3:32:48</t>
+          <t>2:51:24</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1239,7 +1239,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>17:07:44</t>
+          <t>13:51:28</t>
         </is>
       </c>
     </row>
@@ -1269,7 +1269,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2:16:16</t>
+          <t>1:50:23</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1279,7 +1279,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>19:25:30</t>
+          <t>15:43:21</t>
         </is>
       </c>
     </row>
@@ -1309,7 +1309,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2:54:08</t>
+          <t>2:17:26</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1319,7 +1319,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>22:21:38</t>
+          <t>18:02:47</t>
         </is>
       </c>
     </row>
@@ -1349,7 +1349,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2:54:51</t>
+          <t>2:21:05</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1359,7 +1359,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>25:17:59</t>
+          <t>20:25:22</t>
         </is>
       </c>
     </row>
@@ -1389,7 +1389,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>3:49:16</t>
+          <t>3:04:26</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1399,7 +1399,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>29:08:45</t>
+          <t>23:31:18</t>
         </is>
       </c>
     </row>
@@ -1429,7 +1429,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>0:44:47</t>
+          <t>0:35:05</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>29:53:32</t>
+          <t>24:06:23</t>
         </is>
       </c>
     </row>
@@ -1451,7 +1451,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>target_time</t>
+          <t>athlete_pb</t>
         </is>
       </c>
     </row>
@@ -1475,7 +1475,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>29:29:02</t>
+          <t>23:41:53</t>
         </is>
       </c>
     </row>
@@ -1499,7 +1499,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>29:53:32</t>
+          <t>24:06:23</t>
         </is>
       </c>
     </row>
@@ -1510,7 +1510,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>804</v>
+        <v>894</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
implement sqrt adjustment to Riegel's formula in library
</commit_message>
<xml_diff>
--- a/results/tgt_2026_segment_analysis.xlsx
+++ b/results/tgt_2026_segment_analysis.xlsx
@@ -989,7 +989,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1:29:20</t>
+          <t>2:02:46</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -999,7 +999,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>1:30:20</t>
+          <t>2:03:46</t>
         </is>
       </c>
     </row>
@@ -1029,7 +1029,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>1:50:21</t>
+          <t>2:31:38</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -1039,7 +1039,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>3:22:41</t>
+          <t>4:37:23</t>
         </is>
       </c>
     </row>
@@ -1069,7 +1069,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>1:21:58</t>
+          <t>1:52:38</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -1079,7 +1079,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>4:47:39</t>
+          <t>6:33:02</t>
         </is>
       </c>
     </row>
@@ -1109,7 +1109,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2:25:38</t>
+          <t>3:20:08</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>7:16:17</t>
+          <t>9:56:10</t>
         </is>
       </c>
     </row>
@@ -1149,7 +1149,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1:49:56</t>
+          <t>2:31:04</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -1159,7 +1159,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>9:08:13</t>
+          <t>12:29:13</t>
         </is>
       </c>
     </row>
@@ -1189,7 +1189,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1:44:51</t>
+          <t>2:24:05</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1199,7 +1199,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>10:58:04</t>
+          <t>14:58:19</t>
         </is>
       </c>
     </row>
@@ -1229,7 +1229,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2:51:24</t>
+          <t>3:55:31</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1239,7 +1239,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>13:51:28</t>
+          <t>18:55:50</t>
         </is>
       </c>
     </row>
@@ -1269,7 +1269,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>1:50:23</t>
+          <t>2:31:41</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1279,7 +1279,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>15:43:21</t>
+          <t>21:29:01</t>
         </is>
       </c>
     </row>
@@ -1309,7 +1309,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2:17:26</t>
+          <t>3:08:51</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1319,7 +1319,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>18:02:47</t>
+          <t>24:39:52</t>
         </is>
       </c>
     </row>
@@ -1349,7 +1349,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2:21:05</t>
+          <t>3:13:52</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1359,7 +1359,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>20:25:22</t>
+          <t>27:55:14</t>
         </is>
       </c>
     </row>
@@ -1389,7 +1389,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>3:04:26</t>
+          <t>4:13:27</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1399,7 +1399,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>23:31:18</t>
+          <t>32:10:11</t>
         </is>
       </c>
     </row>
@@ -1429,7 +1429,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>0:35:05</t>
+          <t>0:48:12</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>24:06:23</t>
+          <t>32:58:23</t>
         </is>
       </c>
     </row>
@@ -1475,7 +1475,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>23:41:53</t>
+          <t>32:33:53</t>
         </is>
       </c>
     </row>
@@ -1499,7 +1499,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>24:06:23</t>
+          <t>32:58:23</t>
         </is>
       </c>
     </row>
@@ -1510,7 +1510,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>894</v>
+        <v>688</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
time calculator bassed on inverse-GAP conversion
</commit_message>
<xml_diff>
--- a/results/tgt_2026_segment_analysis.xlsx
+++ b/results/tgt_2026_segment_analysis.xlsx
@@ -989,7 +989,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2:02:46</t>
+          <t>1:51:55</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -999,7 +999,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2:03:46</t>
+          <t>1:52:55</t>
         </is>
       </c>
     </row>
@@ -1029,7 +1029,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2:31:38</t>
+          <t>2:18:14</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -1039,7 +1039,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>4:37:23</t>
+          <t>4:13:08</t>
         </is>
       </c>
     </row>
@@ -1069,7 +1069,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>1:52:38</t>
+          <t>1:42:41</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -1079,7 +1079,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>6:33:02</t>
+          <t>5:58:49</t>
         </is>
       </c>
     </row>
@@ -1109,7 +1109,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>3:20:08</t>
+          <t>3:02:27</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>9:56:10</t>
+          <t>9:04:16</t>
         </is>
       </c>
     </row>
@@ -1149,7 +1149,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2:31:04</t>
+          <t>2:17:42</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -1159,7 +1159,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>12:29:13</t>
+          <t>11:23:59</t>
         </is>
       </c>
     </row>
@@ -1189,7 +1189,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2:24:05</t>
+          <t>2:11:21</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1199,7 +1199,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>14:58:19</t>
+          <t>13:40:20</t>
         </is>
       </c>
     </row>
@@ -1229,7 +1229,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>3:55:31</t>
+          <t>3:34:42</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1239,7 +1239,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>18:55:50</t>
+          <t>17:17:02</t>
         </is>
       </c>
     </row>
@@ -1269,7 +1269,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2:31:41</t>
+          <t>2:18:16</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1279,7 +1279,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>21:29:01</t>
+          <t>19:36:49</t>
         </is>
       </c>
     </row>
@@ -1309,7 +1309,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>3:08:51</t>
+          <t>2:52:10</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1319,7 +1319,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>24:39:52</t>
+          <t>22:30:58</t>
         </is>
       </c>
     </row>
@@ -1349,7 +1349,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>3:13:52</t>
+          <t>2:56:44</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1359,7 +1359,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>27:55:14</t>
+          <t>25:29:12</t>
         </is>
       </c>
     </row>
@@ -1389,7 +1389,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>4:13:27</t>
+          <t>3:51:03</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1399,7 +1399,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>32:10:11</t>
+          <t>29:21:45</t>
         </is>
       </c>
     </row>
@@ -1429,7 +1429,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>0:48:12</t>
+          <t>0:43:57</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>32:58:23</t>
+          <t>30:05:42</t>
         </is>
       </c>
     </row>
@@ -1475,7 +1475,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>32:33:53</t>
+          <t>29:41:12</t>
         </is>
       </c>
     </row>
@@ -1499,7 +1499,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>32:58:23</t>
+          <t>30:05:42</t>
         </is>
       </c>
     </row>
@@ -1510,7 +1510,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>688</v>
+        <v>748</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated inverse GAP curve in libraries to reflect ocnstant vertical speed beyond a certain grade
</commit_message>
<xml_diff>
--- a/results/tgt_2026_segment_analysis.xlsx
+++ b/results/tgt_2026_segment_analysis.xlsx
@@ -989,7 +989,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1:51:55</t>
+          <t>2:03:46</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -999,7 +999,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>1:52:55</t>
+          <t>2:04:46</t>
         </is>
       </c>
     </row>
@@ -1029,7 +1029,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2:18:14</t>
+          <t>2:21:46</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -1039,7 +1039,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>4:13:08</t>
+          <t>4:28:32</t>
         </is>
       </c>
     </row>
@@ -1069,7 +1069,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>1:42:41</t>
+          <t>1:48:15</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -1079,7 +1079,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>5:58:49</t>
+          <t>6:19:46</t>
         </is>
       </c>
     </row>
@@ -1109,7 +1109,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>3:02:27</t>
+          <t>3:07:02</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>9:04:16</t>
+          <t>9:29:49</t>
         </is>
       </c>
     </row>
@@ -1149,7 +1149,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2:17:42</t>
+          <t>2:17:45</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -1159,7 +1159,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>11:23:59</t>
+          <t>11:49:34</t>
         </is>
       </c>
     </row>
@@ -1189,7 +1189,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2:11:21</t>
+          <t>2:14:23</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1199,7 +1199,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>13:40:20</t>
+          <t>14:08:57</t>
         </is>
       </c>
     </row>
@@ -1229,7 +1229,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>3:34:42</t>
+          <t>3:41:36</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1239,7 +1239,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>17:17:02</t>
+          <t>17:52:33</t>
         </is>
       </c>
     </row>
@@ -1269,7 +1269,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2:18:16</t>
+          <t>2:24:44</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1279,7 +1279,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>19:36:49</t>
+          <t>20:18:46</t>
         </is>
       </c>
     </row>
@@ -1309,7 +1309,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2:52:10</t>
+          <t>2:52:12</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1319,7 +1319,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>22:30:58</t>
+          <t>23:12:59</t>
         </is>
       </c>
     </row>
@@ -1349,7 +1349,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2:56:44</t>
+          <t>2:58:51</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1359,7 +1359,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>25:29:12</t>
+          <t>26:13:20</t>
         </is>
       </c>
     </row>
@@ -1389,7 +1389,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>3:51:03</t>
+          <t>4:02:35</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1399,7 +1399,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>29:21:45</t>
+          <t>30:17:25</t>
         </is>
       </c>
     </row>
@@ -1429,7 +1429,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>0:43:57</t>
+          <t>0:42:54</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>30:05:42</t>
+          <t>31:00:19</t>
         </is>
       </c>
     </row>
@@ -1475,7 +1475,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>29:41:12</t>
+          <t>30:35:49</t>
         </is>
       </c>
     </row>
@@ -1499,7 +1499,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>30:05:42</t>
+          <t>31:00:19</t>
         </is>
       </c>
     </row>
@@ -1510,7 +1510,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>748</v>
+        <v>728</v>
       </c>
     </row>
   </sheetData>

</xml_diff>